<commit_message>
Added new RDF data schemes and visual schemes, fixed XLSX spreadsheets for economy-table60-64
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table60.xlsx
+++ b/sources/table_normalization/xlsx/economy-table60.xlsx
@@ -115,11 +115,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="5">
-    <numFmt numFmtId="168" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
-    <numFmt numFmtId="169" formatCode="0.0"/>
-    <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="171" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="172" formatCode="_-* #,##0.00\ [$₽-419]_-;\-* #,##0.00\ [$₽-419]_-;_-* &quot;-&quot;??\ [$₽-419]_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="168" formatCode="_-* #,##0.00\ [$₽-419]_-;\-* #,##0.00\ [$₽-419]_-;_-* &quot;-&quot;??\ [$₽-419]_-;_-@_-"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -494,7 +494,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="3" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="1" fontId="7" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -506,7 +506,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="1" fontId="7" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -551,7 +551,7 @@
     <xf numFmtId="1" fontId="8" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="8" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -564,56 +564,44 @@
     <xf numFmtId="1" fontId="8" fillId="0" borderId="6" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="8" fillId="0" borderId="6" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="6" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="170" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="6" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="8" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="8" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="171" fontId="8" fillId="0" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="170" fontId="8" fillId="0" borderId="6" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="6" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="8" fillId="0" borderId="6" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="6" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="171" fontId="8" fillId="0" borderId="12" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="12" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="3" fillId="0" borderId="8" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="8" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="2" fillId="0" borderId="8" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="8" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="172" fontId="2" fillId="0" borderId="13" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="13" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -631,16 +619,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="3" fillId="3" borderId="8" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="3" fillId="3" borderId="8" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="4" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -656,17 +644,29 @@
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="170" fontId="1" fillId="4" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="1" fillId="4" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="171" fontId="6" fillId="4" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="6" fillId="4" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="2" fillId="4" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="4" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -920,8 +920,8 @@
         <xdr:to>
           <xdr:col>2</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>2</xdr:row>
-          <xdr:rowOff>495300</xdr:rowOff>
+          <xdr:row>3</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -979,7 +979,7 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>1181100</xdr:colOff>
+          <xdr:colOff>647700</xdr:colOff>
           <xdr:row>30</xdr:row>
           <xdr:rowOff>342900</xdr:rowOff>
         </xdr:to>
@@ -1306,27 +1306,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="31">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="60" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="2"/>
-      <c r="D1" s="59" t="s">
+      <c r="D1" s="55" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="15"/>
       <c r="F1" s="16"/>
       <c r="G1" s="17"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="37"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
       <c r="J1" s="29"/>
-      <c r="K1" s="60" t="s">
+      <c r="K1" s="57" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="60"/>
+      <c r="L1" s="57"/>
     </row>
     <row r="2" spans="1:12" ht="17">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="59" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="1"/>
@@ -1338,46 +1338,46 @@
       <c r="H2" s="4"/>
       <c r="I2" s="30"/>
       <c r="J2" s="30"/>
-      <c r="K2" s="38" t="s">
+      <c r="K2" s="58" t="s">
         <v>4</v>
       </c>
-      <c r="L2" s="38"/>
+      <c r="L2" s="58"/>
     </row>
     <row r="3" spans="1:12" ht="39">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="48" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="53" t="s">
+      <c r="B3" s="49" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="54" t="s">
+      <c r="C3" s="50" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="54" t="s">
+      <c r="D3" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="55" t="s">
+      <c r="E3" s="51" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="56" t="s">
+      <c r="F3" s="52" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="53" t="s">
+      <c r="G3" s="49" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="54" t="s">
+      <c r="H3" s="50" t="s">
         <v>12</v>
       </c>
-      <c r="I3" s="57" t="s">
+      <c r="I3" s="53" t="s">
         <v>13</v>
       </c>
-      <c r="J3" s="57" t="s">
+      <c r="J3" s="53" t="s">
         <v>14</v>
       </c>
-      <c r="K3" s="58" t="s">
+      <c r="K3" s="54" t="s">
         <v>15</v>
       </c>
-      <c r="L3" s="58" t="s">
+      <c r="L3" s="54" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2428,23 +2428,23 @@
       </c>
     </row>
     <row r="31" spans="1:12" ht="31">
-      <c r="A31" s="49"/>
-      <c r="B31" s="44"/>
-      <c r="C31" s="45"/>
-      <c r="D31" s="46"/>
-      <c r="E31" s="47"/>
+      <c r="A31" s="45"/>
+      <c r="B31" s="40"/>
+      <c r="C31" s="41"/>
+      <c r="D31" s="42"/>
+      <c r="E31" s="43"/>
       <c r="F31" s="28"/>
-      <c r="G31" s="48"/>
-      <c r="H31" s="50"/>
-      <c r="I31" s="51" t="s">
+      <c r="G31" s="44"/>
+      <c r="H31" s="46"/>
+      <c r="I31" s="47" t="s">
         <v>23</v>
       </c>
-      <c r="J31" s="41"/>
-      <c r="K31" s="42">
+      <c r="J31" s="37"/>
+      <c r="K31" s="38">
         <f>SUM(K4:K30)</f>
         <v>9727.5</v>
       </c>
-      <c r="L31" s="43">
+      <c r="L31" s="39">
         <f>SUM(L4:L30)</f>
         <v>2279.8249999999998</v>
       </c>

</xml_diff>